<commit_message>
updates fro mSIRIUS1 testing
</commit_message>
<xml_diff>
--- a/check-target-net/src/cursor_grading_web/wwwroot/uploads/companies_graded.xlsx
+++ b/check-target-net/src/cursor_grading_web/wwwroot/uploads/companies_graded.xlsx
@@ -5426,505 +5426,139 @@
     <x:t>Builds custom advanced manufacturing systems with a focus on high-speed assembly, test, and inspection of automotive electronics components</x:t>
   </x:si>
   <x:si>
-    <x:t>Manufactures automotive wire harnesses, sensors, and electronic modules; likely has in-house R&amp;D and test engineering to validate designs and ensure quality.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Company lists in-house design, manufacturing, and testing capabilities, indicating need for test equipment.</x:t>
+    <x:t>Manufactures automotive wire harnesses and sensors, indicating in-house test/quality control functions that require test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Site explicitly lists 'testing' as a core capability alongside design and manufacturing of electronics, indicating in-house test engineers.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Automotive supplier of seating and electrical systems; no clear evidence of in-house electronic test or R&amp;D labs that would use oscilloscopes or similar equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>No clear evidence of in-house electronic test or measurement work, just metal foil processing.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>States parts undergo advanced testing (vibration, thermal shock) but unclear if they have in-house labs or just resell sensors; no explicit engineering/R&amp;D team mentioned.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: HTTP 301 Moved Permanently</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: Network error: The SSL connection could not be established, see inner exception. (The remote certificate is invalid according to the validation procedure: RemoteCertificateNameMismatch)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Manufactures electronic components like voltage regulators and rectifiers, implying in-house production testing with equipment like oscilloscopes or power supplies.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: HTTP 403 Forbidden</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Manufactures LED lighting and smart trailer systems, implying in-house electronics R&amp;D and testing.</x:t>
   </x:si>
   <x:si>
     <x:t>Scrape failed: Request timed out after 15s</x:t>
   </x:si>
   <x:si>
-    <x:t>Scrape failed: HTTP 403 Forbidden</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Insufficient website content to determine if they have in-house electronics test or engineering functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: The SSL connection could not be established, see inner exception.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: HTTP 301 Moved Permanently</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer of electronic automotive components (voltage regulators, rectifiers), but no direct evidence of in-house test engineering, R&amp;D, or calibration lab visible in the scraped content.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Repairs and remanufactures automotive electronic modules, which likely requires in-house testing and diagnostic equipment like oscilloscopes and power supplies.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house design and manufacturing of electronic LED lighting and smart vehicle systems implies use of test equipment for development and quality assurance.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No clear evidence of in-house electronic testing or engineering; they process metal foils for thermal management applications.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are a retail installer of automotive electronics with no evidence of in-house engineering or test work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>provides in-house electronic repair and calibration services requiring test equipment like oscilloscopes and signal generators</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Website markets automotive electronics but provides no concrete evidence of in-house engineering, R&amp;D, or test lab.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design, develop, and manufacture automotive electronic components and wiring harnesses, implying in-house R&amp;D and test functions that use test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Consumer brand for car audio, no evidence of in-house engineering or test; may only resell/install finished products.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures automotive electronic components (sensors, ignition, fuel injection) and has an Engineered Solutions division, indicating in-house engineering and testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures automotive wiring and components but no clear evidence of in-house electronic test or R&amp;D lab.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No indication of in-house engineering or test; seems to sell and install finished camera products.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides mobile vehicle electronics diagnostics and calibration services, uses specialized automotive tools, but unclear need for general-purpose test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They install and maintain emergency vehicle electronics but show no clear signs of on-site engineering or use of test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They perform in-house repair, remanufacturing, and calibration of automotive electronics, indicating they likely use test equipment like oscilloscopes and meters.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They remanufacture electronic automotive components (e.g., engine control modules, throttle bodies) and mention calibration and repair, indicating in-house electronics testing and diagnostics.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures its own electronic throttle controllers, implying in-house R&amp;D and likely use of test equipment for development and compliance testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures vehicle electronic components, implying in-house engineering and testing labs that use test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped website content is garbled and unreadable, preventing any determination of in-house engineering or test equipment usage.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer of electronic performance components, likely has in-house R&amp;D needing test gear.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MTCA R&amp;D center and multiple manufacturing plants show in-house engineering and testing of electronic automotive systems.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Develops and produces stamped connectors; unclear if they perform in-house electronic testing requiring oscilloscopes or signal generators.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures electronic control units and ADAS, indicating in-house R&amp;D and test.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house engineering and rigorous testing (PPAP, FMEA) on wire harnesses indicates staff who plausibly use test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sells aftermarket automotive electronics but no evidence of in-house engineering, R&amp;D, or test/repair functions visible in website content.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and tests custom ECUs and diagnostic hardware, indicating in-house electronics engineering lab work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sells programmed engine modules but shows no evidence of in-house hardware engineering or general test equipment use; likely relies on automotive-specific programmers.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Full-cycle electronics remanufacturing of automotive electronics implies in-house testing and diagnostics that require test &amp; measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures only mechanical automotive components, no evidence of in-house electronics testing, calibration, or repair work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions 'deep engineering expertise' and 'Engineering Products' but no explicit in-house test/measurement or calibration functions visible in the scraped text.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Company engineers and manufactures automotive electronics, indicating likely use of test equipment for R&amp;D and quality control.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Automotive components manufacturer with no clear indication of in-house electronic R&amp;D or testing functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are a tier-one automotive lighting supplier with in-house engineering and manufacturing, indicating they likely use electronic test equipment for R&amp;D and production testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>The Plymouth, MI location 'specializes in the development and testing' of LED lighting solutions, indicating in-house R&amp;D that likely uses test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Develops advanced sensors, radar systems, and electronic safety components, indicating in-house R&amp;D and test engineering.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Automotive tuning shop; no evidence of in-house electronics engineering or test that would require oscilloscopes or similar gear.</x:t>
+    <x:t>Repair and refurbishment of automotive electronic control units likely requires in-house use of test equipment like oscilloscopes and power supplies.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scraped content shows product categories but no evidence of in-house engineering or test lab; they design/integrate automotive electronics but it's unclear if they own test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Only consumer-facing sales of finished car audio products visible; no evidence of in-house engineering, R&amp;D, or test labs on this page.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: HTTP 429 Too Many Requests</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Performs in-house repair and calibration of electronic instrument clusters, PCMs, and modules, requiring electronic test and measurement equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>In-house design, development, and manufacturing of automotive electronics and wiring harnesses likely requires test equipment for validation and quality assurance.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: HTTP 520 &lt;none&gt;</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Installs finished auto electronics (alarms, audio) with no evidence of in-house engineering, testing, or repair that requires T&amp;M equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Site suggests product development but no clear evidence of in-house engineering or test hardware usage.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Manufactures electronic automotive parts (sensors, engine management) at their engineering and manufacturing facilities, indicating in-house R&amp;D and testing.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>In-house manufacturing and development of electronic components like wire harnesses and battery sensors requires R&amp;D and test equipment such as oscilloscopes and power supplies.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Performs in-house repair, remanufacturing, calibration, and testing of automotive electronics, indicating use of test equipment like oscilloscopes and signal generators.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>They design, develop, and manufacture automotive electronics, ECUs, and provide testing services; their MxSuite integrates with test equipment, indicating in-house use of measurement gear.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Primarily installs finished electronic components into vehicles, with no visible in-house engineering or test lab for electronic diagnostics.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Provides vehicle electronics diagnostics and calibration services, but not clear if they use general-purpose test equipment; likely uses specialized automotive tools.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>They remanufacture electronic control modules and perform calibration, indicating in-house test and diagnostic work on electronic hardware.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Site shows they design and sell automotive performance electronics but no clear evidence of in-house engineering lab or test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: Network error: The SSL connection could not be established, see inner exception. (The remote certificate is invalid according to the validation procedure: RemoteCertificateNameMismatch, RemoteCertificateChainErrors)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Develops and produces connectors; development may involve testing, but no explicit test/engineering lab or equipment use is evident.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MTCA R&amp;D center develops ADAS and infotainment systems, and manufacturing includes hybrid battery modules, indicating in-house electronic testing and calibration.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: Network error: An error occurred while sending the request. (The response ended prematurely. (ResponseEnded))</x:t>
+  </x:si>
+  <x:si>
+    <x:t>U.S. manufacturer of electronic control systems; likely has in-house R&amp;D/engineering that uses test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Designs and manufactures electronic systems, implying in-house R&amp;D and testing that requires test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scraped text shows deep engineering expertise and custom manufacturing, suggesting in-house electronic design and testing.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scrape failed: HTTP 502 Bad Gateway</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sells pre-programmed automotive control modules and offers reprogramming, but no clear evidence of in-house engineering or hardware-level diagnostics requiring test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FlexStation-IOT ECU test station and custom ECU development indicate in-house hardware engineering likely using test and measurement equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Describes in-house engineering and manufacturing of automotive electronics, implying need for test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Primarily mechanical component manufacturer; no evidence of in-house electronics testing or R&amp;D requiring test equipment.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Installs finished vehicle electronics, no visible engineering or test function.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Primarily resells and installs aftermarket automotive accessories, no indication of in-house engineering or testing</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Automotive lighting manufacturer with in-house engineering and R&amp;D, likely using test equipment for design and validation of electronic lighting components.</x:t>
   </x:si>
   <x:si>
     <x:t>Scrape failed: Page body was empty after parsing</x:t>
   </x:si>
   <x:si>
-    <x:t>Mentions R&amp;D, advanced electronics, sensor tech, and design of electromagnetic valves, indicating in-house engineering likely using test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They perform in-house PCB assembly, EMS, and ODM with engineering support, likely using test equipment for quality control.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions product development and engineering centers, likely involving design and testing of automotive electronic components.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Installs and resells finished automotive electronics; no evidence of in-house engineering, calibration, or repair work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are an engineering and manufacturing company with a technical center, likely having engineers who test and develop automotive systems and machine tools, requiring electronic test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>insufficient scraped content to determine if they have in-house engineering/test functions</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures electronic controls, motors, and TPMS/EHPS/PEPS systems, indicating in-house R&amp;D and testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Company has in-house engineering and testing lab for automotive electronic components, performing electrical testing per SAE standards.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house design, engineering and testing of EV powertrain systems including motor controllers, battery management, and VCU programming, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vertically integrated electronic manufacturer with in-house engineering and ISO 9001-2015 certification suggests need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house development and engineering of OBD tuning software and hardware, plus design and manufacturing of performance parts, suggest need for electronic test and measurement.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They engineer proprietary sensor/control systems, implying in-house R&amp;D and testing that would require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are a vehicle upfitter and distributor of finished public safety equipment (lights, sirens, barriers); no evidence of in-house engineering, R&amp;D, or test functions that would require T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They remanufacture and repair electronic instrument clusters, implying in-house electronics diagnostics and repair requiring test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Technical resource for vehicle wiring installations and module configurations, but no evidence of in-house engineering, R&amp;D, or repair work requiring test &amp; measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures modular electronic assemblies and automotive lighting products, very likely requiring in-house test, validation, or quality control with electronic test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They list 'Testing' as a capability and manufacture electronic components and wire harnesses, typically requiring in-house electronic test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: HTTP 406 Not Acceptable</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Remanufactures mechanical fuel system components; no clear evidence of in-house electronic test or diagnostics that would require general-purpose T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides a software platform for electronics manufacturing inspection and test data, but no clear evidence of in-house hardware engineering, repair, or calibration work requiring test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions integrated modules for control units and power electronics, but website text focuses on plastic molding and assembly with no clear evidence of in-house electronic testing or engineering labs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and tests power control modules, with advanced testing indicating in-house engineering.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content is insufficient to determine if they have in-house engineering or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer with R&amp;D, but no evidence of electronic testing or equipment need.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Trade association focused on software OTA standards, no evidence of in-house electronic hardware testing, engineering, or manufacturing that would require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures automotive semiconductors and ECUs, indicating in-house design and testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mechatronics products imply potential electronic testing, but no clear evidence of using T&amp;M equipment like oscilloscopes.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures automotive LED lighting, suggesting possible in-house electronics engineering and testing, but no explicit mention of test equipment or calibration labs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content insufficient to determine if they perform in-house electronic test/engineering work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: The requested name is valid, but no data of the requested type was found. (omron.com:443)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No evidence of in-house test/engineering; purely a wholesale warehouse distributor of auto parts, chemicals, and oils.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Automotive parts supplier with no visible electronic engineering, R&amp;D, or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Engineering and prototyping lab that develops products from concept to testing, implying in-house use of test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content shows automotive chemical products, no indication of in-house electronics engineering or repair that would need test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tier 1 automotive supplier with manufacturing and custom tool development, but no mention of in-house electronic test or diagnostics; unclear if they have engineers using T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures electronic transmission controllers in-house, with custom engineering and tuning, implying use of test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>No evidence of in-house electronic engineering, R&amp;D, or repair; company focuses on automotive mechanical tools and training.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: The requested name is valid, but no data of the requested type was found. (shinko.co.jp:443)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house design and manufacturing of advanced electrical connectors and harness systems strongly implies engineering teams that need to validate, test, and troubleshoot electronic hardware with instruments like oscilloscopes and meters.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Resells automotive diagnostic tools including lab scopes, but no clear evidence of in-house engineering, calibration, or repair work; appears primarily a reseller.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions custom design, but unclear if they do in-house electronic testing versus just assembling or reselling automotive equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Develops, engineers, and manufactures its own LED emergency lighting products, implying an internal R&amp;D and test function that likely uses electronic test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They install aftermarket vehicle electronics but no evidence of in-house engineering or test equipment use; primarily an installation service.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design, develop, and manufacture electronic solutions with in-house R&amp;D, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers PCBA and full box-build with engineering services, indicating in-house test and measurement needs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides Engineering &amp; Design Services and manufactures PCBA and electronic components, implying in-house testing and diagnostics using test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer custom electronic hardware design, prototyping, and production support with 20 years of engineering experience, indicating in-house engineers who use test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content was insufficient to make a determination</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures hydraulic brake calipers and components; no indication of electronic testing or engineering lab on site.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures PCBs, RF components, and mission systems, implying in-house engineering and testing requiring oscilloscopes, signal generators, etc.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They perform functional testing, in-circuit testing, and have AOI and 3D X-ray inspection, indicating in-house engineering/test work on electronic hardware.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers electronic circuit troubleshooting, repair, design, and testing services, indicating in-house need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Distributor of electronic components; mentions test &amp; measurement products but no evidence of in-house engineering or test work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Curtis has in-house R&amp;D, engineering, and manufacturing of motor controllers and battery management systems, indicating they likely use test equipment like oscilloscopes and power supplies.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer of automotive chemical additives; no indication of in-house electronics engineering, testing, or repair; likely no need for test &amp; measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures mechatronic and actuator systems, implying potential in-house electronic engineering and testing, but scraped content lacks explicit mention of test labs or T&amp;M equipment usage.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures high-frequency ceramic components, indicating in-house R&amp;D and testing that likely uses RF test equipment like spectrum analyzers and network analyzers.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: The requested name is valid, but no data of the requested type was found. (hosiden.com:443)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer's representative for electronic components, no evidence of in-house engineering, testing, or repair functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They provide PCB coating services, but no clear evidence of in-house electronic engineering or test functions that would require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>scraped content only shows generic marketing language, no mention of engineering, R&amp;D, or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions developing products from ground up and extensive testing tailored to application, indicating in-house engineering/R&amp;D that likely requires test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: The requested name is valid, but no data of the requested type was found. (foster-electric.com:443)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PCB manufacturer implies some in-house testing, but no explicit mention of test equipment, engineering, or R&amp;D functions that would need oscilloscopes, signal generators, etc.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMS company performing PCB assembly, likely has in-house test and debug engineers who use test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design and manufacture electronic components (sensors, LED lighting, power distribution) with in-house R&amp;D and labs, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Makes connectors for ECUs and sensors, but site emphasizes mechanical manufacturing (casting, stamping) without indication of electronic test or engineering.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMS provider with in-house engineering, testing (DFT), PCB assembly, and repair depot, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cohu designs and manufactures semiconductor test equipment, indicating in-house R&amp;D and engineering teams that use test and measurement instruments for development and validation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures custom motor and motion control systems, indicating in-house engineering and testing of electronic hardware.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures power semiconductors (Si, SiC, GaN), MOSFETs, and digital isolators, implying in-house R&amp;D and test labs requiring oscilloscopes, signal generators, and other T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides PCB design and manufacturing but no explicit mention of in-house test, calibration, or repair work on electronic hardware.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Contract manufacturer offering PCBA, box build, testing, and repair services, indicating in-house use of test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturers' sales representative firm offering technical sales and engineering support, but no indication of in-house testing, repair, or R&amp;D labs that would use T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mechanical parts manufacturer with no visible in-house electronic engineering or test function requiring T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer in-house test engineering, design, and manufacturing services, clearly needing T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer's rep providing engineering support, but no evidence of in-house test/measurement lab or hardware engineering.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMS provider with in-house design engineering and high-volume PCBA manufacturing, implying test and quality control using T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They manufacture automotive electronic components like ECUs and sensors, have inspection/measuring equipment, and operate smart factories, indicating in-house R&amp;D and testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Contract manufacturer of precision mechanical components, no evidence of in-house electronic engineering or test work that would require T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Electronics contract manufacturer with in-house assembly, testing to IPC standards, design, and reverse-engineering, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions 'Advanced Test Engineering' and performs PCBA-to-complete electronic modules manufacture, indicating in-house testing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They perform in-house PCB assembly and antenna design with engineering support, requiring test and measurement equipment for quality assurance.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house rigorous performance testing and analytical testing services for laminate materials likely require electronic test equipment for characterization.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are a distributor of electronic components, not a manufacturer; no clear evidence of in-house engineering or testing labs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers turnkey manufacturing, design, and engineering services involving electronic hardware, indicating in-house test and measurement needs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers in-house embedded hardware design, PCB layout, prototype testing, and hardware calibration, requiring oscilloscopes and other T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Develops boundary-scan test hardware and software, clearly has in-house engineering and testing functions that require test &amp; measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Develops and applies nano coatings for electronics protection but no clear evidence of in-house electronic testing, R&amp;D, or engineering teams using T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Consumer car audio sales site, no visible in-house engineering, repair, or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design and manufacture vehicle safety electronics and subject them to rigorous testing, indicating an in-house engineering and test function that likely requires test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers in-house electronics manufacturing services including assembly, testing, engineering support, and depot repair, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Engineering services explicitly include testing and prototyping, indicating in-house use of test equipment for complex electronics manufacturing.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mentions product development and engineering of LED lighting controls, suggesting possible in-house electronics design, but no explicit evidence of test equipment usage.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures components with in-house R&amp;D and testing, clearly employs engineers who need test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They are a manufacturer's representative, and while they mention technical expertise and engineering solutions, there is no clear evidence of in-house test, calibration, or repair work that would require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design and manufacture flexible circuits in-house for mission-critical applications, implying need for electrical testing equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs electronic hardware for 3D printers but no explicit evidence of in-house test/calibration work on electronics, only general manufacturing and services mentioned.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures automated programming systems, indicating in-house engineering and hardware testing requiring test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>In-house engineering, PCB assembly, system integration, and functional testing indicate active use of test and measurement equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and manufactures their own automated test systems, implying in-house engineering and testing teams.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer in-house PCB design and electronics manufacturing services, indicating engineering and test functions that require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scrape failed: Network error: No connection could be made because the target machine actively refused it. (jebconet.com:443)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures custom magnetics and electronic assemblies with in-house rigorous testing (thermal shock, dielectric, corona) and holds AS9100D certification, indicating need for test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Makes electro-mechanical assemblies and wire harnesses, but scraped text shows no explicit in-house engineering, test, or calibration functions that would clearly require oscilloscopes or signal generators.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers design, prototyping, and box-build integration services, indicating in-house engineering that likely uses test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design and manufacture electronic controllers and displays, implying in-house engineering and test functions that require test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sheldahl designs and manufactures flexible circuits and printed electronics, requiring in-house engineering and testing of electronic hardware, as evidenced by their R&amp;D collaboration, innovation videos, and custom solutions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides electronic manufacturing services with in-house test capabilities likely requiring oscilloscopes and power supplies.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They apply conformal coatings to electronics but no evidence of in-house electronic testing, repair, or R&amp;D that would require oscilloscopes or similar T&amp;M gear.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer contract manufacturing with electrical assembly and extensive testing protocols, likely requiring oscilloscopes and other test gear.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer electronics testing and design-for-test services, indicating in-house use of test equipment like oscilloscopes and signal generators.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They design and test custom electromagnetic components (coils, solenoids, relays) in-house, with dedicated testing labs, indicating a need for electronic test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content only shows JavaScript requirement message, no meaningful company information available.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Offers PCB assembly and test services, and designs OEM electronic products, indicating in-house engineering and test functions likely requiring oscilloscopes, signal generators, and power supplies.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>They offer remanufacturing and repair services for automotive and consumer electronics, indicating in-house diagnostic and repair work requiring test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufacturer sales rep firm providing technical sales and marketing, no evidence of in-house engineering or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Designs and builds custom test and inspection systems for automotive electronics, implying in-house engineering likely using test equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scraped content only shows consumer goods categories, no evidence of in-house engineering or test functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Provides mechanical manufacturing services to electronics industry but no evidence of in-house electronic test or engineering functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sells optical inspection systems and does metal fabrication, but no clear evidence of in-house electronic test, repair, or R&amp;D using T&amp;M equipment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Manufactures magnetic components for automotive electronics, implying some R&amp;D and production testing, but scraped text lacks explicit mention of in-house test/measurement functions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PCB manufacturer with engineering support and DFM feedback, but no clear evidence of in-house electronic testing or use of oscilloscopes/signal generators.</x:t>
+    <x:t>Scrape failed: Cancelled by user</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -7297,10 +6931,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M24" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="N24" s="0" t="s">
-        <x:v>1803</x:v>
+        <x:v>1805</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -7341,10 +6975,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M25" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="N25" s="0" t="s">
-        <x:v>1805</x:v>
+        <x:v>1803</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -7388,7 +7022,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N26" s="0" t="s">
-        <x:v>1811</x:v>
+        <x:v>1804</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -7432,7 +7066,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N27" s="0" t="s">
-        <x:v>1804</x:v>
+        <x:v>1811</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -7473,7 +7107,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M28" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N28" s="0" t="s">
         <x:v>1808</x:v>
@@ -7564,7 +7198,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N30" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1807</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -7608,7 +7242,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N31" s="0" t="s">
-        <x:v>1807</x:v>
+        <x:v>1806</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -7652,7 +7286,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N32" s="0" t="s">
-        <x:v>1809</x:v>
+        <x:v>1812</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -7696,7 +7330,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N33" s="0" t="s">
-        <x:v>1804</x:v>
+        <x:v>1809</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -7740,7 +7374,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N34" s="0" t="s">
-        <x:v>1816</x:v>
+        <x:v>1814</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -7784,7 +7418,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N35" s="0" t="s">
-        <x:v>1814</x:v>
+        <x:v>1813</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -7828,7 +7462,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N36" s="0" t="s">
-        <x:v>1812</x:v>
+        <x:v>1819</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -7869,7 +7503,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N37" s="0" t="s">
-        <x:v>1813</x:v>
+        <x:v>1816</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -7913,7 +7547,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N38" s="0" t="s">
-        <x:v>1815</x:v>
+        <x:v>1817</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -7957,7 +7591,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N39" s="0" t="s">
-        <x:v>1817</x:v>
+        <x:v>1821</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -8001,7 +7635,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N40" s="0" t="s">
-        <x:v>1819</x:v>
+        <x:v>1820</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -8045,7 +7679,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N41" s="0" t="s">
-        <x:v>1807</x:v>
+        <x:v>1806</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -8083,10 +7717,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M42" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N42" s="0" t="s">
-        <x:v>1824</x:v>
+        <x:v>1815</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -8127,10 +7761,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M43" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N43" s="0" t="s">
-        <x:v>1818</x:v>
+        <x:v>1822</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -8174,7 +7808,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N44" s="0" t="s">
-        <x:v>1820</x:v>
+        <x:v>1826</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -8215,10 +7849,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M45" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N45" s="0" t="s">
-        <x:v>1825</x:v>
+        <x:v>1818</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -8259,7 +7893,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N46" s="0" t="s">
-        <x:v>1821</x:v>
+        <x:v>1825</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -8300,10 +7934,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M47" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N47" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1824</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -8347,7 +7981,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N48" s="0" t="s">
-        <x:v>1829</x:v>
+        <x:v>1830</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -8385,10 +8019,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M49" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="N49" s="0" t="s">
-        <x:v>1827</x:v>
+        <x:v>1828</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -8429,7 +8063,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N50" s="0" t="s">
-        <x:v>1822</x:v>
+        <x:v>1823</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -8473,7 +8107,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N51" s="0" t="s">
-        <x:v>1823</x:v>
+        <x:v>1827</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -8517,7 +8151,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N52" s="0" t="s">
-        <x:v>1828</x:v>
+        <x:v>1831</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -8561,7 +8195,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N53" s="0" t="s">
-        <x:v>1804</x:v>
+        <x:v>1811</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -8602,10 +8236,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M54" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N54" s="0" t="s">
-        <x:v>1826</x:v>
+        <x:v>1833</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -8649,7 +8283,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N55" s="0" t="s">
-        <x:v>1832</x:v>
+        <x:v>1842</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:14" x14ac:dyDescent="0.25">
@@ -8687,10 +8321,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M56" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N56" s="0" t="s">
-        <x:v>1837</x:v>
+        <x:v>1835</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -8734,7 +8368,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N57" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1811</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -8778,7 +8412,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N58" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1829</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:14" x14ac:dyDescent="0.25">
@@ -8822,7 +8456,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N59" s="0" t="s">
-        <x:v>1838</x:v>
+        <x:v>1839</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -8863,10 +8497,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M60" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N60" s="0" t="s">
-        <x:v>1831</x:v>
+        <x:v>1832</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:14" x14ac:dyDescent="0.25">
@@ -8948,7 +8582,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N62" s="0" t="s">
-        <x:v>1834</x:v>
+        <x:v>1837</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:14" x14ac:dyDescent="0.25">
@@ -8992,7 +8626,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N63" s="0" t="s">
-        <x:v>1830</x:v>
+        <x:v>1834</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:14" x14ac:dyDescent="0.25">
@@ -9033,7 +8667,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N64" s="0" t="s">
-        <x:v>1803</x:v>
+        <x:v>1815</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -9077,7 +8711,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N65" s="0" t="s">
-        <x:v>1833</x:v>
+        <x:v>1838</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:14" x14ac:dyDescent="0.25">
@@ -9121,7 +8755,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N66" s="0" t="s">
-        <x:v>1836</x:v>
+        <x:v>1840</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -9161,12 +8795,6 @@
       <x:c r="L67" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M67" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N67" s="0" t="s">
-        <x:v>1843</x:v>
-      </x:c>
     </x:row>
     <x:row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A68" s="0" t="s">
@@ -9206,10 +8834,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M68" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N68" s="0" t="s">
-        <x:v>1835</x:v>
+        <x:v>1818</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:14" x14ac:dyDescent="0.25">
@@ -9253,7 +8881,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="N69" s="0" t="s">
-        <x:v>1848</x:v>
+        <x:v>1841</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -9294,10 +8922,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="M70" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N70" s="0" t="s">
-        <x:v>1839</x:v>
+        <x:v>1836</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:14" x14ac:dyDescent="0.25">
@@ -9341,7 +8969,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N71" s="0" t="s">
-        <x:v>1840</x:v>
+        <x:v>1843</x:v>
       </x:c>
     </x:row>
     <x:row r="72" spans="1:14" x14ac:dyDescent="0.25">
@@ -9381,12 +9009,6 @@
       <x:c r="L72" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M72" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N72" s="0" t="s">
-        <x:v>1842</x:v>
-      </x:c>
     </x:row>
     <x:row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A73" s="0" t="s">
@@ -9426,10 +9048,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M73" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N73" s="0" t="s">
-        <x:v>1841</x:v>
+        <x:v>1818</x:v>
       </x:c>
     </x:row>
     <x:row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -9469,12 +9091,6 @@
       <x:c r="L74" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M74" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N74" s="0" t="s">
-        <x:v>1846</x:v>
-      </x:c>
     </x:row>
     <x:row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A75" s="0" t="s">
@@ -9513,12 +9129,6 @@
       <x:c r="L75" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M75" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N75" s="0" t="s">
-        <x:v>1845</x:v>
-      </x:c>
     </x:row>
     <x:row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A76" s="0" t="s">
@@ -9557,12 +9167,6 @@
       <x:c r="L76" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M76" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N76" s="0" t="s">
-        <x:v>1854</x:v>
-      </x:c>
     </x:row>
     <x:row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A77" s="0" t="s">
@@ -9602,10 +9206,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M77" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N77" s="0" t="s">
-        <x:v>1855</x:v>
+        <x:v>1815</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:14" x14ac:dyDescent="0.25">
@@ -9645,12 +9249,6 @@
       <x:c r="L78" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M78" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N78" s="0" t="s">
-        <x:v>1847</x:v>
-      </x:c>
     </x:row>
     <x:row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A79" s="0" t="s">
@@ -9689,12 +9287,6 @@
       <x:c r="L79" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M79" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N79" s="0" t="s">
-        <x:v>1850</x:v>
-      </x:c>
     </x:row>
     <x:row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A80" s="0" t="s">
@@ -9733,12 +9325,6 @@
       <x:c r="L80" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M80" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N80" s="0" t="s">
-        <x:v>1849</x:v>
-      </x:c>
     </x:row>
     <x:row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A81" s="0" t="s">
@@ -9777,12 +9363,6 @@
       <x:c r="L81" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M81" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N81" s="0" t="s">
-        <x:v>1857</x:v>
-      </x:c>
     </x:row>
     <x:row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A82" s="0" t="s">
@@ -9869,7 +9449,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N83" s="0" t="s">
-        <x:v>1804</x:v>
+        <x:v>1809</x:v>
       </x:c>
     </x:row>
     <x:row r="84" spans="1:14" x14ac:dyDescent="0.25">
@@ -9909,12 +9489,6 @@
       <x:c r="L84" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M84" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N84" s="0" t="s">
-        <x:v>1852</x:v>
-      </x:c>
     </x:row>
     <x:row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A85" s="0" t="s">
@@ -9950,12 +9524,6 @@
       <x:c r="L85" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M85" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N85" s="0" t="s">
-        <x:v>1851</x:v>
-      </x:c>
     </x:row>
     <x:row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A86" s="0" t="s">
@@ -9994,12 +9562,6 @@
       <x:c r="L86" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M86" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N86" s="0" t="s">
-        <x:v>1853</x:v>
-      </x:c>
     </x:row>
     <x:row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A87" s="0" t="s">
@@ -10035,12 +9597,6 @@
       <x:c r="L87" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M87" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N87" s="0" t="s">
-        <x:v>1859</x:v>
-      </x:c>
     </x:row>
     <x:row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A88" s="0" t="s">
@@ -10077,10 +9633,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="M88" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N88" s="0" t="s">
-        <x:v>1863</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="89" spans="1:14" x14ac:dyDescent="0.25">
@@ -10118,10 +9674,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="M89" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N89" s="0" t="s">
-        <x:v>1858</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -10159,10 +9715,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M90" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N90" s="0" t="s">
-        <x:v>1856</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -10203,7 +9759,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N91" s="0" t="s">
-        <x:v>1803</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="92" spans="1:14" x14ac:dyDescent="0.25">
@@ -10241,10 +9797,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M92" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N92" s="0" t="s">
-        <x:v>1860</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="93" spans="1:14" x14ac:dyDescent="0.25">
@@ -10285,10 +9841,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M93" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N93" s="0" t="s">
-        <x:v>1869</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="94" spans="1:14" x14ac:dyDescent="0.25">
@@ -10332,7 +9888,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N94" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="95" spans="1:14" x14ac:dyDescent="0.25">
@@ -10373,10 +9929,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M95" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N95" s="0" t="s">
-        <x:v>1870</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -10420,7 +9976,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N96" s="0" t="s">
-        <x:v>1806</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="97" spans="1:14" x14ac:dyDescent="0.25">
@@ -10461,10 +10017,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M97" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N97" s="0" t="s">
-        <x:v>1865</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="98" spans="1:14" x14ac:dyDescent="0.25">
@@ -10505,10 +10061,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M98" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N98" s="0" t="s">
-        <x:v>1864</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="99" spans="1:14" x14ac:dyDescent="0.25">
@@ -10549,10 +10105,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M99" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N99" s="0" t="s">
-        <x:v>1866</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="100" spans="1:14" x14ac:dyDescent="0.25">
@@ -10593,10 +10149,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M100" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N100" s="0" t="s">
-        <x:v>1861</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="101" spans="1:14" x14ac:dyDescent="0.25">
@@ -10640,7 +10196,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N101" s="0" t="s">
-        <x:v>1867</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="102" spans="1:14" x14ac:dyDescent="0.25">
@@ -10684,7 +10240,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N102" s="0" t="s">
-        <x:v>1803</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="103" spans="1:14" x14ac:dyDescent="0.25">
@@ -10728,7 +10284,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N103" s="0" t="s">
-        <x:v>1875</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="104" spans="1:14" x14ac:dyDescent="0.25">
@@ -10772,7 +10328,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N104" s="0" t="s">
-        <x:v>1881</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="105" spans="1:14" x14ac:dyDescent="0.25">
@@ -10812,12 +10368,6 @@
       <x:c r="L105" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M105" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N105" s="0" t="s">
-        <x:v>1872</x:v>
-      </x:c>
     </x:row>
     <x:row r="106" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A106" s="0" t="s">
@@ -10856,12 +10406,6 @@
       <x:c r="L106" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M106" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N106" s="0" t="s">
-        <x:v>1862</x:v>
-      </x:c>
     </x:row>
     <x:row r="107" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A107" s="0" t="s">
@@ -10900,12 +10444,6 @@
       <x:c r="L107" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M107" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N107" s="0" t="s">
-        <x:v>1803</x:v>
-      </x:c>
     </x:row>
     <x:row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A108" s="0" t="s">
@@ -10944,12 +10482,6 @@
       <x:c r="L108" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M108" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N108" s="0" t="s">
-        <x:v>1871</x:v>
-      </x:c>
     </x:row>
     <x:row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A109" s="0" t="s">
@@ -10988,12 +10520,6 @@
       <x:c r="L109" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M109" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N109" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="110" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A110" s="0" t="s">
@@ -11032,12 +10558,6 @@
       <x:c r="L110" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M110" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N110" s="0" t="s">
-        <x:v>1876</x:v>
-      </x:c>
     </x:row>
     <x:row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A111" s="0" t="s">
@@ -11076,12 +10596,6 @@
       <x:c r="L111" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M111" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N111" s="0" t="s">
-        <x:v>1873</x:v>
-      </x:c>
     </x:row>
     <x:row r="112" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A112" s="0" t="s">
@@ -11120,12 +10634,6 @@
       <x:c r="L112" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M112" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N112" s="0" t="s">
-        <x:v>1868</x:v>
-      </x:c>
     </x:row>
     <x:row r="113" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A113" s="0" t="s">
@@ -11164,12 +10672,6 @@
       <x:c r="L113" s="0" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="M113" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N113" s="0" t="s">
-        <x:v>1899</x:v>
-      </x:c>
     </x:row>
     <x:row r="114" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A114" s="0" t="s">
@@ -11208,12 +10710,6 @@
       <x:c r="L114" s="0" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="M114" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N114" s="0" t="s">
-        <x:v>1878</x:v>
-      </x:c>
     </x:row>
     <x:row r="115" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A115" s="0" t="s">
@@ -11252,12 +10748,6 @@
       <x:c r="L115" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M115" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N115" s="0" t="s">
-        <x:v>1879</x:v>
-      </x:c>
     </x:row>
     <x:row r="116" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A116" s="0" t="s">
@@ -11296,12 +10786,6 @@
       <x:c r="L116" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M116" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N116" s="0" t="s">
-        <x:v>1844</x:v>
-      </x:c>
     </x:row>
     <x:row r="117" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A117" s="0" t="s">
@@ -11340,12 +10824,6 @@
       <x:c r="L117" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M117" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N117" s="0" t="s">
-        <x:v>1885</x:v>
-      </x:c>
     </x:row>
     <x:row r="118" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A118" s="0" t="s">
@@ -11381,12 +10859,6 @@
       <x:c r="L118" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M118" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N118" s="0" t="s">
-        <x:v>1886</x:v>
-      </x:c>
     </x:row>
     <x:row r="119" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A119" s="0" t="s">
@@ -11425,12 +10897,6 @@
       <x:c r="L119" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M119" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N119" s="0" t="s">
-        <x:v>1880</x:v>
-      </x:c>
     </x:row>
     <x:row r="120" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A120" s="0" t="s">
@@ -11469,12 +10935,6 @@
       <x:c r="L120" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M120" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N120" s="0" t="s">
-        <x:v>1893</x:v>
-      </x:c>
     </x:row>
     <x:row r="121" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A121" s="0" t="s">
@@ -11513,12 +10973,6 @@
       <x:c r="L121" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M121" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N121" s="0" t="s">
-        <x:v>1877</x:v>
-      </x:c>
     </x:row>
     <x:row r="122" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A122" s="0" t="s">
@@ -11554,12 +11008,6 @@
       <x:c r="L122" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M122" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N122" s="0" t="s">
-        <x:v>1874</x:v>
-      </x:c>
     </x:row>
     <x:row r="123" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A123" s="0" t="s">
@@ -11595,12 +11043,6 @@
       <x:c r="L123" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M123" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N123" s="0" t="s">
-        <x:v>1884</x:v>
-      </x:c>
     </x:row>
     <x:row r="124" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A124" s="0" t="s">
@@ -11639,12 +11081,6 @@
       <x:c r="L124" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M124" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N124" s="0" t="s">
-        <x:v>1883</x:v>
-      </x:c>
     </x:row>
     <x:row r="125" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A125" s="0" t="s">
@@ -11680,12 +11116,6 @@
       <x:c r="L125" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M125" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N125" s="0" t="s">
-        <x:v>1887</x:v>
-      </x:c>
     </x:row>
     <x:row r="126" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A126" s="0" t="s">
@@ -11722,10 +11152,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M126" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N126" s="0" t="s">
-        <x:v>1888</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="127" spans="1:14" x14ac:dyDescent="0.25">
@@ -11765,12 +11195,6 @@
       <x:c r="L127" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M127" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N127" s="0" t="s">
-        <x:v>1904</x:v>
-      </x:c>
     </x:row>
     <x:row r="128" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A128" s="0" t="s">
@@ -11809,12 +11233,6 @@
       <x:c r="L128" s="0" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="M128" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N128" s="0" t="s">
-        <x:v>1903</x:v>
-      </x:c>
     </x:row>
     <x:row r="129" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A129" s="0" t="s">
@@ -11853,12 +11271,6 @@
       <x:c r="L129" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M129" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N129" s="0" t="s">
-        <x:v>1894</x:v>
-      </x:c>
     </x:row>
     <x:row r="130" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A130" s="0" t="s">
@@ -11897,12 +11309,6 @@
       <x:c r="L130" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M130" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N130" s="0" t="s">
-        <x:v>1900</x:v>
-      </x:c>
     </x:row>
     <x:row r="131" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A131" s="0" t="s">
@@ -11942,10 +11348,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M131" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N131" s="0" t="s">
-        <x:v>1890</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="132" spans="1:14" x14ac:dyDescent="0.25">
@@ -11985,12 +11391,6 @@
       <x:c r="L132" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M132" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N132" s="0" t="s">
-        <x:v>1889</x:v>
-      </x:c>
     </x:row>
     <x:row r="133" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A133" s="0" t="s">
@@ -12029,12 +11429,6 @@
       <x:c r="L133" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M133" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N133" s="0" t="s">
-        <x:v>1882</x:v>
-      </x:c>
     </x:row>
     <x:row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A134" s="0" t="s">
@@ -12073,12 +11467,6 @@
       <x:c r="L134" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M134" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N134" s="0" t="s">
-        <x:v>1905</x:v>
-      </x:c>
     </x:row>
     <x:row r="135" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A135" s="0" t="s">
@@ -12117,12 +11505,6 @@
       <x:c r="L135" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M135" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N135" s="0" t="s">
-        <x:v>1891</x:v>
-      </x:c>
     </x:row>
     <x:row r="136" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A136" s="0" t="s">
@@ -12161,12 +11543,6 @@
       <x:c r="L136" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M136" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N136" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="137" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A137" s="0" t="s">
@@ -12205,12 +11581,6 @@
       <x:c r="L137" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M137" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N137" s="0" t="s">
-        <x:v>1897</x:v>
-      </x:c>
     </x:row>
     <x:row r="138" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A138" s="0" t="s">
@@ -12249,12 +11619,6 @@
       <x:c r="L138" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M138" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N138" s="0" t="s">
-        <x:v>1911</x:v>
-      </x:c>
     </x:row>
     <x:row r="139" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A139" s="0" t="s">
@@ -12294,10 +11658,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="M139" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N139" s="0" t="s">
-        <x:v>1895</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="140" spans="1:14" x14ac:dyDescent="0.25">
@@ -12337,12 +11701,6 @@
       <x:c r="L140" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M140" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N140" s="0" t="s">
-        <x:v>1913</x:v>
-      </x:c>
     </x:row>
     <x:row r="141" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A141" s="0" t="s">
@@ -12381,12 +11739,6 @@
       <x:c r="L141" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M141" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N141" s="0" t="s">
-        <x:v>1896</x:v>
-      </x:c>
     </x:row>
     <x:row r="142" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A142" s="0" t="s">
@@ -12429,7 +11781,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="N142" s="0" t="s">
-        <x:v>1892</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="143" spans="1:14" x14ac:dyDescent="0.25">
@@ -12469,12 +11821,6 @@
       <x:c r="L143" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M143" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N143" s="0" t="s">
-        <x:v>1898</x:v>
-      </x:c>
     </x:row>
     <x:row r="144" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A144" s="0" t="s">
@@ -12513,12 +11859,6 @@
       <x:c r="L144" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M144" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N144" s="0" t="s">
-        <x:v>1909</x:v>
-      </x:c>
     </x:row>
     <x:row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A145" s="0" t="s">
@@ -12557,12 +11897,6 @@
       <x:c r="L145" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M145" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N145" s="0" t="s">
-        <x:v>1908</x:v>
-      </x:c>
     </x:row>
     <x:row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A146" s="0" t="s">
@@ -12601,12 +11935,6 @@
       <x:c r="L146" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M146" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N146" s="0" t="s">
-        <x:v>1901</x:v>
-      </x:c>
     </x:row>
     <x:row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A147" s="0" t="s">
@@ -12646,10 +11974,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="M147" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="N147" s="0" t="s">
-        <x:v>1919</x:v>
+        <x:v>1845</x:v>
       </x:c>
     </x:row>
     <x:row r="148" spans="1:14" x14ac:dyDescent="0.25">
@@ -12689,12 +12017,6 @@
       <x:c r="L148" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M148" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N148" s="0" t="s">
-        <x:v>1906</x:v>
-      </x:c>
     </x:row>
     <x:row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A149" s="0" t="s">
@@ -12733,12 +12055,6 @@
       <x:c r="L149" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M149" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N149" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A150" s="0" t="s">
@@ -12777,12 +12093,6 @@
       <x:c r="L150" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M150" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N150" s="0" t="s">
-        <x:v>1912</x:v>
-      </x:c>
     </x:row>
     <x:row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A151" s="0" t="s">
@@ -12821,12 +12131,6 @@
       <x:c r="L151" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M151" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N151" s="0" t="s">
-        <x:v>1916</x:v>
-      </x:c>
     </x:row>
     <x:row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A152" s="0" t="s">
@@ -12865,12 +12169,6 @@
       <x:c r="L152" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M152" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N152" s="0" t="s">
-        <x:v>1915</x:v>
-      </x:c>
     </x:row>
     <x:row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A153" s="0" t="s">
@@ -12909,12 +12207,6 @@
       <x:c r="L153" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M153" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N153" s="0" t="s">
-        <x:v>1910</x:v>
-      </x:c>
     </x:row>
     <x:row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A154" s="0" t="s">
@@ -12953,12 +12245,6 @@
       <x:c r="L154" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M154" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N154" s="0" t="s">
-        <x:v>1929</x:v>
-      </x:c>
     </x:row>
     <x:row r="155" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A155" s="0" t="s">
@@ -12997,12 +12283,6 @@
       <x:c r="L155" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M155" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N155" s="0" t="s">
-        <x:v>1918</x:v>
-      </x:c>
     </x:row>
     <x:row r="156" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A156" s="0" t="s">
@@ -13041,12 +12321,6 @@
       <x:c r="L156" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M156" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N156" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="157" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A157" s="0" t="s">
@@ -13085,12 +12359,6 @@
       <x:c r="L157" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M157" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N157" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="158" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A158" s="0" t="s">
@@ -13129,12 +12397,6 @@
       <x:c r="L158" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M158" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N158" s="0" t="s">
-        <x:v>1902</x:v>
-      </x:c>
     </x:row>
     <x:row r="159" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A159" s="0" t="s">
@@ -13173,12 +12435,6 @@
       <x:c r="L159" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M159" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N159" s="0" t="s">
-        <x:v>1844</x:v>
-      </x:c>
     </x:row>
     <x:row r="160" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A160" s="0" t="s">
@@ -13217,12 +12473,6 @@
       <x:c r="L160" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M160" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N160" s="0" t="s">
-        <x:v>1921</x:v>
-      </x:c>
     </x:row>
     <x:row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A161" s="0" t="s">
@@ -13261,12 +12511,6 @@
       <x:c r="L161" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M161" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N161" s="0" t="s">
-        <x:v>1907</x:v>
-      </x:c>
     </x:row>
     <x:row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A162" s="0" t="s">
@@ -13305,12 +12549,6 @@
       <x:c r="L162" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M162" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N162" s="0" t="s">
-        <x:v>1923</x:v>
-      </x:c>
     </x:row>
     <x:row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A163" s="0" t="s">
@@ -13349,12 +12587,6 @@
       <x:c r="L163" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M163" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N163" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A164" s="0" t="s">
@@ -13393,12 +12625,6 @@
       <x:c r="L164" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M164" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N164" s="0" t="s">
-        <x:v>1924</x:v>
-      </x:c>
     </x:row>
     <x:row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A165" s="0" t="s">
@@ -13437,12 +12663,6 @@
       <x:c r="L165" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M165" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N165" s="0" t="s">
-        <x:v>1914</x:v>
-      </x:c>
     </x:row>
     <x:row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A166" s="0" t="s">
@@ -13481,12 +12701,6 @@
       <x:c r="L166" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M166" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N166" s="0" t="s">
-        <x:v>1922</x:v>
-      </x:c>
     </x:row>
     <x:row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A167" s="0" t="s">
@@ -13525,12 +12739,6 @@
       <x:c r="L167" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M167" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N167" s="0" t="s">
-        <x:v>1917</x:v>
-      </x:c>
     </x:row>
     <x:row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A168" s="0" t="s">
@@ -13569,12 +12777,6 @@
       <x:c r="L168" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M168" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N168" s="0" t="s">
-        <x:v>1928</x:v>
-      </x:c>
     </x:row>
     <x:row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A169" s="0" t="s">
@@ -13613,12 +12815,6 @@
       <x:c r="L169" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M169" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N169" s="0" t="s">
-        <x:v>1926</x:v>
-      </x:c>
     </x:row>
     <x:row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A170" s="0" t="s">
@@ -13657,12 +12853,6 @@
       <x:c r="L170" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M170" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N170" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A171" s="0" t="s">
@@ -13701,12 +12891,6 @@
       <x:c r="L171" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M171" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N171" s="0" t="s">
-        <x:v>1920</x:v>
-      </x:c>
     </x:row>
     <x:row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A172" s="0" t="s">
@@ -13745,12 +12929,6 @@
       <x:c r="L172" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M172" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N172" s="0" t="s">
-        <x:v>1934</x:v>
-      </x:c>
     </x:row>
     <x:row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A173" s="0" t="s">
@@ -13789,12 +12967,6 @@
       <x:c r="L173" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M173" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N173" s="0" t="s">
-        <x:v>1803</x:v>
-      </x:c>
     </x:row>
     <x:row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A174" s="0" t="s">
@@ -13833,12 +13005,6 @@
       <x:c r="L174" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M174" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N174" s="0" t="s">
-        <x:v>1931</x:v>
-      </x:c>
     </x:row>
     <x:row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A175" s="0" t="s">
@@ -13877,12 +13043,6 @@
       <x:c r="L175" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M175" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N175" s="0" t="s">
-        <x:v>1925</x:v>
-      </x:c>
     </x:row>
     <x:row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A176" s="0" t="s">
@@ -13921,12 +13081,6 @@
       <x:c r="L176" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M176" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N176" s="0" t="s">
-        <x:v>1844</x:v>
-      </x:c>
     </x:row>
     <x:row r="177" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A177" s="0" t="s">
@@ -13965,12 +13119,6 @@
       <x:c r="L177" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M177" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N177" s="0" t="s">
-        <x:v>1938</x:v>
-      </x:c>
     </x:row>
     <x:row r="178" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A178" s="0" t="s">
@@ -14009,12 +13157,6 @@
       <x:c r="L178" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M178" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N178" s="0" t="s">
-        <x:v>1927</x:v>
-      </x:c>
     </x:row>
     <x:row r="179" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A179" s="0" t="s">
@@ -14053,12 +13195,6 @@
       <x:c r="L179" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M179" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N179" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="180" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A180" s="0" t="s">
@@ -14097,12 +13233,6 @@
       <x:c r="L180" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M180" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N180" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="181" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A181" s="0" t="s">
@@ -14141,12 +13271,6 @@
       <x:c r="L181" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M181" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N181" s="0" t="s">
-        <x:v>1932</x:v>
-      </x:c>
     </x:row>
     <x:row r="182" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A182" s="0" t="s">
@@ -14185,12 +13309,6 @@
       <x:c r="L182" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M182" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N182" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="183" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A183" s="0" t="s">
@@ -14229,12 +13347,6 @@
       <x:c r="L183" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M183" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N183" s="0" t="s">
-        <x:v>1940</x:v>
-      </x:c>
     </x:row>
     <x:row r="184" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A184" s="0" t="s">
@@ -14273,12 +13385,6 @@
       <x:c r="L184" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M184" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N184" s="0" t="s">
-        <x:v>1937</x:v>
-      </x:c>
     </x:row>
     <x:row r="185" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A185" s="0" t="s">
@@ -14317,12 +13423,6 @@
       <x:c r="L185" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M185" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N185" s="0" t="s">
-        <x:v>1930</x:v>
-      </x:c>
     </x:row>
     <x:row r="186" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A186" s="0" t="s">
@@ -14361,12 +13461,6 @@
       <x:c r="L186" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M186" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N186" s="0" t="s">
-        <x:v>1942</x:v>
-      </x:c>
     </x:row>
     <x:row r="187" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A187" s="0" t="s">
@@ -14405,12 +13499,6 @@
       <x:c r="L187" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M187" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N187" s="0" t="s">
-        <x:v>1941</x:v>
-      </x:c>
     </x:row>
     <x:row r="188" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A188" s="0" t="s">
@@ -14449,12 +13537,6 @@
       <x:c r="L188" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M188" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N188" s="0" t="s">
-        <x:v>1803</x:v>
-      </x:c>
     </x:row>
     <x:row r="189" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A189" s="0" t="s">
@@ -14493,12 +13575,6 @@
       <x:c r="L189" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M189" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N189" s="0" t="s">
-        <x:v>1933</x:v>
-      </x:c>
     </x:row>
     <x:row r="190" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A190" s="0" t="s">
@@ -14537,12 +13613,6 @@
       <x:c r="L190" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M190" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N190" s="0" t="s">
-        <x:v>1935</x:v>
-      </x:c>
     </x:row>
     <x:row r="191" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A191" s="0" t="s">
@@ -14581,12 +13651,6 @@
       <x:c r="L191" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M191" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N191" s="0" t="s">
-        <x:v>1945</x:v>
-      </x:c>
     </x:row>
     <x:row r="192" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A192" s="0" t="s">
@@ -14625,12 +13689,6 @@
       <x:c r="L192" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M192" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N192" s="0" t="s">
-        <x:v>1939</x:v>
-      </x:c>
     </x:row>
     <x:row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A193" s="0" t="s">
@@ -14669,12 +13727,6 @@
       <x:c r="L193" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M193" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N193" s="0" t="s">
-        <x:v>1944</x:v>
-      </x:c>
     </x:row>
     <x:row r="194" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A194" s="0" t="s">
@@ -14713,12 +13765,6 @@
       <x:c r="L194" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M194" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N194" s="0" t="s">
-        <x:v>1943</x:v>
-      </x:c>
     </x:row>
     <x:row r="195" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A195" s="0" t="s">
@@ -14757,12 +13803,6 @@
       <x:c r="L195" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M195" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N195" s="0" t="s">
-        <x:v>1967</x:v>
-      </x:c>
     </x:row>
     <x:row r="196" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A196" s="0" t="s">
@@ -14801,12 +13841,6 @@
       <x:c r="L196" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M196" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N196" s="0" t="s">
-        <x:v>1936</x:v>
-      </x:c>
     </x:row>
     <x:row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A197" s="0" t="s">
@@ -14845,12 +13879,6 @@
       <x:c r="L197" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M197" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N197" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="198" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A198" s="0" t="s">
@@ -14889,12 +13917,6 @@
       <x:c r="L198" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M198" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N198" s="0" t="s">
-        <x:v>1954</x:v>
-      </x:c>
     </x:row>
     <x:row r="199" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A199" s="0" t="s">
@@ -14933,12 +13955,6 @@
       <x:c r="L199" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M199" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N199" s="0" t="s">
-        <x:v>1950</x:v>
-      </x:c>
     </x:row>
     <x:row r="200" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A200" s="0" t="s">
@@ -14977,12 +13993,6 @@
       <x:c r="L200" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M200" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N200" s="0" t="s">
-        <x:v>1946</x:v>
-      </x:c>
     </x:row>
     <x:row r="201" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A201" s="0" t="s">
@@ -15021,12 +14031,6 @@
       <x:c r="L201" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M201" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N201" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="202" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A202" s="0" t="s">
@@ -15065,12 +14069,6 @@
       <x:c r="L202" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M202" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N202" s="0" t="s">
-        <x:v>1948</x:v>
-      </x:c>
     </x:row>
     <x:row r="203" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A203" s="0" t="s">
@@ -15109,12 +14107,6 @@
       <x:c r="L203" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M203" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N203" s="0" t="s">
-        <x:v>1949</x:v>
-      </x:c>
     </x:row>
     <x:row r="204" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A204" s="0" t="s">
@@ -15153,12 +14145,6 @@
       <x:c r="L204" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M204" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N204" s="0" t="s">
-        <x:v>1953</x:v>
-      </x:c>
     </x:row>
     <x:row r="205" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A205" s="0" t="s">
@@ -15197,12 +14183,6 @@
       <x:c r="L205" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M205" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N205" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A206" s="0" t="s">
@@ -15241,12 +14221,6 @@
       <x:c r="L206" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M206" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N206" s="0" t="s">
-        <x:v>1963</x:v>
-      </x:c>
     </x:row>
     <x:row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A207" s="0" t="s">
@@ -15285,12 +14259,6 @@
       <x:c r="L207" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M207" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N207" s="0" t="s">
-        <x:v>1955</x:v>
-      </x:c>
     </x:row>
     <x:row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A208" s="0" t="s">
@@ -15329,12 +14297,6 @@
       <x:c r="L208" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M208" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N208" s="0" t="s">
-        <x:v>1952</x:v>
-      </x:c>
     </x:row>
     <x:row r="209" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A209" s="0" t="s">
@@ -15373,12 +14335,6 @@
       <x:c r="L209" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M209" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N209" s="0" t="s">
-        <x:v>1951</x:v>
-      </x:c>
     </x:row>
     <x:row r="210" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A210" s="0" t="s">
@@ -15417,12 +14373,6 @@
       <x:c r="L210" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M210" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N210" s="0" t="s">
-        <x:v>1806</x:v>
-      </x:c>
     </x:row>
     <x:row r="211" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A211" s="0" t="s">
@@ -15461,12 +14411,6 @@
       <x:c r="L211" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M211" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N211" s="0" t="s">
-        <x:v>1956</x:v>
-      </x:c>
     </x:row>
     <x:row r="212" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A212" s="0" t="s">
@@ -15505,12 +14449,6 @@
       <x:c r="L212" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M212" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N212" s="0" t="s">
-        <x:v>1804</x:v>
-      </x:c>
     </x:row>
     <x:row r="213" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A213" s="0" t="s">
@@ -15549,12 +14487,6 @@
       <x:c r="L213" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M213" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N213" s="0" t="s">
-        <x:v>1961</x:v>
-      </x:c>
     </x:row>
     <x:row r="214" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A214" s="0" t="s">
@@ -15593,12 +14525,6 @@
       <x:c r="L214" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M214" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N214" s="0" t="s">
-        <x:v>1965</x:v>
-      </x:c>
     </x:row>
     <x:row r="215" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A215" s="0" t="s">
@@ -15637,12 +14563,6 @@
       <x:c r="L215" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M215" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N215" s="0" t="s">
-        <x:v>1960</x:v>
-      </x:c>
     </x:row>
     <x:row r="216" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A216" s="0" t="s">
@@ -15681,12 +14601,6 @@
       <x:c r="L216" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M216" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N216" s="0" t="s">
-        <x:v>1959</x:v>
-      </x:c>
     </x:row>
     <x:row r="217" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A217" s="0" t="s">
@@ -15725,12 +14639,6 @@
       <x:c r="L217" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M217" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N217" s="0" t="s">
-        <x:v>1957</x:v>
-      </x:c>
     </x:row>
     <x:row r="218" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A218" s="0" t="s">
@@ -15769,12 +14677,6 @@
       <x:c r="L218" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M218" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N218" s="0" t="s">
-        <x:v>1947</x:v>
-      </x:c>
     </x:row>
     <x:row r="219" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A219" s="0" t="s">
@@ -15813,12 +14715,6 @@
       <x:c r="L219" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="M219" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N219" s="0" t="s">
-        <x:v>1964</x:v>
-      </x:c>
     </x:row>
     <x:row r="220" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A220" s="0" t="s">
@@ -15857,12 +14753,6 @@
       <x:c r="L220" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M220" s="0" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="N220" s="0" t="s">
-        <x:v>1966</x:v>
-      </x:c>
     </x:row>
     <x:row r="221" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A221" s="0" t="s">
@@ -15901,12 +14791,6 @@
       <x:c r="L221" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M221" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N221" s="0" t="s">
-        <x:v>1958</x:v>
-      </x:c>
     </x:row>
     <x:row r="222" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A222" s="0" t="s">
@@ -15945,12 +14829,6 @@
       <x:c r="L222" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="M222" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="N222" s="0" t="s">
-        <x:v>1803</x:v>
-      </x:c>
     </x:row>
     <x:row r="223" spans="1:14" x14ac:dyDescent="0.25">
       <x:c r="A223" s="0" t="s">
@@ -15988,12 +14866,6 @@
       </x:c>
       <x:c r="L223" s="0" t="s">
         <x:v>23</x:v>
-      </x:c>
-      <x:c r="M223" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N223" s="0" t="s">
-        <x:v>1962</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>